<commit_message>
Handle fallback logic functions
</commit_message>
<xml_diff>
--- a/data/Jun/InternalDailyReport_Jun.xlsx
+++ b/data/Jun/InternalDailyReport_Jun.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Jun\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD9BB75B-8B12-410E-8ED3-558496620576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB3724FA-9F09-4A99-96A8-B025244C26A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="1000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="1000" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="19" r:id="rId1"/>
@@ -29055,7 +29055,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A2:R88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -29128,7 +29127,7 @@
       </c>
       <c r="Q2" s="15"/>
     </row>
-    <row r="3" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="15"/>
       <c r="B3" s="15" t="s">
         <v>26</v>
@@ -29172,7 +29171,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="15"/>
       <c r="B4" s="15" t="s">
         <v>26</v>
@@ -29216,7 +29215,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="15"/>
       <c r="B5" s="15" t="s">
         <v>26</v>
@@ -29260,7 +29259,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="15"/>
       <c r="B6" s="15" t="s">
         <v>26</v>
@@ -29304,7 +29303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="15"/>
       <c r="B7" s="15" t="s">
         <v>26</v>
@@ -29348,7 +29347,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="15"/>
       <c r="B8" s="15" t="s">
         <v>26</v>
@@ -29392,7 +29391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="15"/>
       <c r="B9" s="15" t="s">
         <v>26</v>
@@ -29440,7 +29439,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="15"/>
       <c r="B10" s="15" t="s">
         <v>26</v>
@@ -29484,7 +29483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="15"/>
       <c r="B11" s="15" t="s">
         <v>26</v>
@@ -29528,7 +29527,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="15"/>
       <c r="B12" s="15" t="s">
         <v>26</v>
@@ -29572,7 +29571,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" s="15"/>
       <c r="B13" s="15" t="s">
         <v>26</v>
@@ -29620,7 +29619,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" s="15"/>
       <c r="B14" s="15" t="s">
         <v>26</v>
@@ -29664,7 +29663,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" s="15"/>
       <c r="B15" s="15" t="s">
         <v>26</v>
@@ -29708,7 +29707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" s="15"/>
       <c r="B16" s="15" t="s">
         <v>26</v>
@@ -29756,7 +29755,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="15"/>
       <c r="B17" s="15" t="s">
         <v>26</v>
@@ -29800,7 +29799,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="15"/>
       <c r="B18" s="15" t="s">
         <v>26</v>
@@ -29844,7 +29843,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="15"/>
       <c r="B19" s="15" t="s">
         <v>26</v>
@@ -29892,7 +29891,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" s="15"/>
       <c r="B20" s="15" t="s">
         <v>26</v>
@@ -29936,7 +29935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="15"/>
       <c r="B21" s="15" t="s">
         <v>26</v>
@@ -29980,7 +29979,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" s="15"/>
       <c r="B22" s="15" t="s">
         <v>26</v>
@@ -30028,7 +30027,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" s="15"/>
       <c r="B23" s="15" t="s">
         <v>26</v>
@@ -30072,7 +30071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="15"/>
       <c r="B24" s="15" t="s">
         <v>26</v>
@@ -30116,7 +30115,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
         <v>101</v>
       </c>
@@ -30164,7 +30163,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="26" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
         <v>101</v>
       </c>
@@ -30208,7 +30207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
         <v>101</v>
       </c>
@@ -31032,7 +31031,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="45" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="15"/>
       <c r="B45" s="15" t="s">
         <v>26</v>
@@ -31076,7 +31075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" s="15"/>
       <c r="B46" s="15" t="s">
         <v>26</v>
@@ -31120,7 +31119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47" s="15"/>
       <c r="B47" s="15" t="s">
         <v>26</v>
@@ -31164,7 +31163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" s="15"/>
       <c r="B48" s="15" t="s">
         <v>26</v>
@@ -31208,7 +31207,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" s="15"/>
       <c r="B49" s="15" t="s">
         <v>26</v>
@@ -31258,7 +31257,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="50" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" s="15"/>
       <c r="B50" s="15" t="s">
         <v>26</v>
@@ -31302,7 +31301,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" s="15"/>
       <c r="B51" s="15" t="s">
         <v>26</v>
@@ -31350,7 +31349,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="52" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A52" s="15"/>
       <c r="B52" s="15" t="s">
         <v>26</v>
@@ -31400,7 +31399,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="53" spans="1:18" s="19" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:18" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="17"/>
       <c r="B53" s="17" t="s">
         <v>26</v>
@@ -31450,7 +31449,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="54" spans="1:18" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A54" s="15"/>
       <c r="B54" s="15" t="s">
         <v>26</v>
@@ -31501,15 +31500,15 @@
       </c>
       <c r="G56" s="1">
         <f t="shared" ref="G56:Q56" si="2">SUBTOTAL(9,G3:G54)</f>
-        <v>10215</v>
+        <v>37930</v>
       </c>
       <c r="H56" s="1">
         <f t="shared" si="2"/>
-        <v>500</v>
+        <v>1515</v>
       </c>
       <c r="I56" s="1">
         <f t="shared" si="2"/>
-        <v>9715</v>
+        <v>36415</v>
       </c>
       <c r="J56" s="1">
         <f t="shared" si="2"/>
@@ -31541,7 +31540,7 @@
       </c>
       <c r="Q56" s="1">
         <f t="shared" si="2"/>
-        <v>17</v>
+        <v>52</v>
       </c>
     </row>
     <row r="57" spans="1:18" x14ac:dyDescent="0.25">
@@ -31941,11 +31940,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A2:P54" xr:uid="{00000000-0009-0000-0000-000001000000}">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="c.cuong"/>
-      </filters>
-    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:P54">
       <sortCondition ref="J2:J54"/>
     </sortState>

</xml_diff>